<commit_message>
Cross-check CoStar v2 rent/occ and make pipeline dating drive the forecast
- Parse CoStar v2 Avg Asking/Unit + Vacancy %; keep both sources' occupancy
  and rent side-by-side, choose the displayed value via --occ-source /
  --rent-source (default CoStar), and flag divergence (>=2 pts occ, >=5% rent).
- Reconciliation Log now shows CoStar vs RealPage occ and rent per property.
- Add --pipeline-dates: analyst-supplied delivery quarters for pipeline deals
  flow into the quarterly absorption table at 0% occupancy, lifting
  "% to be absorbed". Each run emits a pipeline_dates template CSV.
- Update example fixtures (CoStar v2, sample pipeline_dates.csv) and SKILL.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/examples/canyon_ridge/CoStar_5mi_50unit_properties.xlsx
+++ b/examples/canyon_ridge/CoStar_5mi_50unit_properties.xlsx
@@ -6,13 +6,13 @@
     <x:workbookView/>
   </x:bookViews>
   <x:sheets>
-    <x:sheet name="Export061926" sheetId="1" r:id="R1ffd4d93f3a0414b"/>
+    <x:sheet name="Export061926" sheetId="1" r:id="R2582b1f8933a4789"/>
   </x:sheets>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="192">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="195">
   <x:si>
     <x:t>Property Name</x:t>
   </x:si>
@@ -78,6 +78,15 @@
   </x:si>
   <x:si>
     <x:t>Submarket Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Avg Asking/SF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Avg Asking/Unit</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Vacancy %</x:t>
   </x:si>
   <x:si>
     <x:t>Carriage Crossing Apartments</x:t>
@@ -594,6 +603,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="3">
+    <x:numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <x:numFmt numFmtId="165" formatCode="$#,##0"/>
+    <x:numFmt numFmtId="166" formatCode="#,##0.0"/>
+  </x:numFmts>
   <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
@@ -629,7 +643,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
@@ -643,6 +657,15 @@
     <x:xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
@@ -653,6 +676,15 @@
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
     <x:xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom"/>
+    </x:xf>
+    <x:xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
   </x:cellXfs>
@@ -949,7 +981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:dimension ref="A1:V34"/>
+  <x:dimension ref="A1:Y34"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="27.140625" style="2" bestFit="1" customWidth="1"/>
@@ -970,94 +1002,106 @@
     <x:col min="19" max="19" width="47.85546875" style="2" bestFit="1" customWidth="1"/>
     <x:col min="20" max="20" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
     <x:col min="21" max="22" width="19.140625" style="2" bestFit="1" customWidth="1"/>
+    <x:col min="23" max="23" width="13.7109375" style="5" bestFit="1" customWidth="1"/>
+    <x:col min="24" max="24" width="15.5703125" style="6" bestFit="1" customWidth="1"/>
+    <x:col min="25" max="25" width="10.5703125" style="7" bestFit="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="6" t="s">
+      <x:c r="A1" s="9" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="s">
+      <x:c r="B1" s="9" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="s">
+      <x:c r="C1" s="9" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="s">
+      <x:c r="D1" s="9" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="s">
+      <x:c r="E1" s="9" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="s">
+      <x:c r="F1" s="9" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G1" s="7" t="s">
+      <x:c r="G1" s="10" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="s">
+      <x:c r="H1" s="9" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="I1" s="8" t="s">
+      <x:c r="I1" s="11" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="J1" s="7" t="s">
+      <x:c r="J1" s="10" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="K1" s="7" t="s">
+      <x:c r="K1" s="10" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="L1" s="7" t="s">
+      <x:c r="L1" s="10" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="M1" s="7" t="s">
+      <x:c r="M1" s="10" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="N1" s="7" t="s">
+      <x:c r="N1" s="10" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="O1" s="7" t="s">
+      <x:c r="O1" s="10" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="P1" s="7" t="s">
+      <x:c r="P1" s="10" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="Q1" s="6" t="s">
+      <x:c r="Q1" s="9" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="R1" s="6" t="s">
+      <x:c r="R1" s="9" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="S1" s="6" t="s">
+      <x:c r="S1" s="9" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="T1" s="6" t="s">
+      <x:c r="T1" s="9" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="U1" s="6" t="s">
+      <x:c r="U1" s="9" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="V1" s="6" t="s">
+      <x:c r="V1" s="9" t="s">
         <x:v>21</x:v>
+      </x:c>
+      <x:c r="W1" s="12" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="X1" s="13" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="Y1" s="14" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="s">
-        <x:v>22</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B2" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G2" s="3">
         <x:v>1990</x:v>
@@ -1081,39 +1125,48 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R2" s="2" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="S2" s="2" t="s">
-        <x:v>29</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="T2" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U2" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V2" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W2" s="5">
+        <x:v>2.31</x:v>
+      </x:c>
+      <x:c r="X2" s="6">
+        <x:v>1847</x:v>
+      </x:c>
+      <x:c r="Y2" s="7">
+        <x:v>1.5152</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="s">
-        <x:v>33</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C3" s="2" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D3" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E3" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F3" s="2" t="s">
-        <x:v>35</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="G3" s="3">
         <x:v>1978</x:v>
@@ -1134,39 +1187,48 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R3" s="2" t="s">
-        <x:v>36</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="S3" s="2" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="T3" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U3" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V3" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="W3" s="5">
+        <x:v>1.73</x:v>
+      </x:c>
+      <x:c r="X3" s="6">
+        <x:v>1371</x:v>
+      </x:c>
+      <x:c r="Y3" s="7">
+        <x:v>1.6393</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D4" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E4" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F4" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G4" s="3">
         <x:v>1972</x:v>
@@ -1184,39 +1246,48 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R4" s="2" t="s">
-        <x:v>41</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="S4" s="2" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="T4" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U4" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V4" s="2" t="s">
-        <x:v>43</x:v>
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="W4" s="5">
+        <x:v>1.47</x:v>
+      </x:c>
+      <x:c r="X4" s="6">
+        <x:v>1401</x:v>
+      </x:c>
+      <x:c r="Y4" s="7">
+        <x:v>14.6853</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="s">
-        <x:v>44</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C5" s="2" t="s">
-        <x:v>45</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D5" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E5" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F5" s="2" t="s">
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="G5" s="3">
         <x:v>1993</x:v>
@@ -1237,39 +1308,45 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R5" s="2" t="s">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="S5" s="2" t="s">
-        <x:v>48</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="T5" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U5" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V5" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="W5" s="5">
+        <x:v>1.55</x:v>
+      </x:c>
+      <x:c r="X5" s="6">
+        <x:v>805</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="s">
-        <x:v>49</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C6" s="2" t="s">
-        <x:v>50</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D6" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E6" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F6" s="2" t="s">
-        <x:v>35</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="G6" s="3">
         <x:v>1995</x:v>
@@ -1293,39 +1370,48 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R6" s="2" t="s">
-        <x:v>51</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="S6" s="2" t="s">
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="T6" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U6" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V6" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="W6" s="5">
+        <x:v>1.43</x:v>
+      </x:c>
+      <x:c r="X6" s="6">
+        <x:v>1426</x:v>
+      </x:c>
+      <x:c r="Y6" s="7">
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2" t="s">
-        <x:v>53</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C7" s="2" t="s">
-        <x:v>54</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D7" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E7" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F7" s="2" t="s">
-        <x:v>55</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G7" s="3">
         <x:v>1993</x:v>
@@ -1349,39 +1435,48 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R7" s="2" t="s">
-        <x:v>56</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="S7" s="2" t="s">
-        <x:v>57</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="T7" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U7" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="V7" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="W7" s="5">
+        <x:v>1.66</x:v>
+      </x:c>
+      <x:c r="X7" s="6">
+        <x:v>1579</x:v>
+      </x:c>
+      <x:c r="Y7" s="7">
+        <x:v>11.6667</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="s">
-        <x:v>60</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C8" s="2" t="s">
-        <x:v>61</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D8" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E8" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F8" s="2" t="s">
-        <x:v>62</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="G8" s="3">
         <x:v>1980</x:v>
@@ -1405,45 +1500,54 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R8" s="2" t="s">
-        <x:v>63</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="S8" s="2" t="s">
-        <x:v>64</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="T8" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U8" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V8" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W8" s="5">
+        <x:v>3.09</x:v>
+      </x:c>
+      <x:c r="X8" s="6">
+        <x:v>1354</x:v>
+      </x:c>
+      <x:c r="Y8" s="7">
+        <x:v>3.4091</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="s">
-        <x:v>65</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C9" s="2" t="s">
-        <x:v>66</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D9" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E9" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F9" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G9" s="3">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="H9" s="2" t="s">
-        <x:v>67</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I9" s="4">
         <x:v>889</x:v>
@@ -1464,39 +1568,48 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="R9" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="S9" s="2" t="s">
-        <x:v>69</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="T9" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U9" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V9" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W9" s="5">
+        <x:v>2.37</x:v>
+      </x:c>
+      <x:c r="X9" s="6">
+        <x:v>2104</x:v>
+      </x:c>
+      <x:c r="Y9" s="7">
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2" t="s">
-        <x:v>70</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C10" s="2" t="s">
-        <x:v>71</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D10" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E10" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F10" s="2" t="s">
-        <x:v>55</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G10" s="3">
         <x:v>1973</x:v>
@@ -1520,39 +1633,48 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R10" s="2" t="s">
-        <x:v>72</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="S10" s="2" t="s">
-        <x:v>73</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="T10" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U10" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="V10" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="W10" s="5">
+        <x:v>1.72</x:v>
+      </x:c>
+      <x:c r="X10" s="6">
+        <x:v>1570</x:v>
+      </x:c>
+      <x:c r="Y10" s="7">
+        <x:v>1.4085</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2" t="s">
-        <x:v>74</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C11" s="2" t="s">
-        <x:v>75</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="D11" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E11" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F11" s="2" t="s">
-        <x:v>76</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="G11" s="3">
         <x:v>1994</x:v>
@@ -1573,39 +1695,48 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R11" s="2" t="s">
-        <x:v>77</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="S11" s="2" t="s">
-        <x:v>78</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="T11" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U11" s="2" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="V11" s="2" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="W11" s="5">
+        <x:v>1.76</x:v>
+      </x:c>
+      <x:c r="X11" s="6">
+        <x:v>2314</x:v>
+      </x:c>
+      <x:c r="Y11" s="7">
+        <x:v>2.027</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="2" t="s">
-        <x:v>80</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C12" s="2" t="s">
-        <x:v>81</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D12" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E12" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F12" s="2" t="s">
-        <x:v>55</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G12" s="3">
         <x:v>2015</x:v>
@@ -1626,42 +1757,51 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q12" s="2" t="s">
-        <x:v>82</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="R12" s="2" t="s">
-        <x:v>82</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="S12" s="2" t="s">
-        <x:v>83</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="T12" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U12" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="V12" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="W12" s="5">
+        <x:v>1.6</x:v>
+      </x:c>
+      <x:c r="X12" s="6">
+        <x:v>1577</x:v>
+      </x:c>
+      <x:c r="Y12" s="7">
+        <x:v>1.4493</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="2" t="s">
-        <x:v>84</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B13" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C13" s="2" t="s">
-        <x:v>85</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D13" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E13" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F13" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G13" s="3">
         <x:v>1995</x:v>
@@ -1685,39 +1825,48 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R13" s="2" t="s">
-        <x:v>51</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="S13" s="2" t="s">
-        <x:v>86</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="T13" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U13" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V13" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W13" s="5">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="X13" s="6">
+        <x:v>1611</x:v>
+      </x:c>
+      <x:c r="Y13" s="7">
+        <x:v>2.0548</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="2" t="s">
-        <x:v>87</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B14" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C14" s="2" t="s">
-        <x:v>88</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D14" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E14" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F14" s="2" t="s">
-        <x:v>89</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="G14" s="3">
         <x:v>1990</x:v>
@@ -1738,45 +1887,54 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R14" s="2" t="s">
-        <x:v>90</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="S14" s="2" t="s">
-        <x:v>91</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="T14" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U14" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V14" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W14" s="5">
+        <x:v>1.7</x:v>
+      </x:c>
+      <x:c r="X14" s="6">
+        <x:v>1682</x:v>
+      </x:c>
+      <x:c r="Y14" s="7">
+        <x:v>4.5455</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="2" t="s">
-        <x:v>92</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B15" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C15" s="2" t="s">
-        <x:v>93</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D15" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E15" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F15" s="2" t="s">
-        <x:v>94</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="G15" s="3">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="H15" s="2" t="s">
-        <x:v>95</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="I15" s="4">
         <x:v>888</x:v>
@@ -1797,42 +1955,51 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q15" s="2" t="s">
-        <x:v>96</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="R15" s="2" t="s">
-        <x:v>97</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="S15" s="2" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="T15" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U15" s="2" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="V15" s="2" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="W15" s="5">
+        <x:v>2.58</x:v>
+      </x:c>
+      <x:c r="X15" s="6">
+        <x:v>2289</x:v>
+      </x:c>
+      <x:c r="Y15" s="7">
+        <x:v>1.0453</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2" t="s">
-        <x:v>99</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B16" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C16" s="2" t="s">
-        <x:v>100</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="D16" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E16" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F16" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G16" s="3">
         <x:v>2002</x:v>
@@ -1856,39 +2023,45 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R16" s="2" t="s">
-        <x:v>101</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="S16" s="2" t="s">
-        <x:v>102</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="T16" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U16" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V16" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W16" s="5">
+        <x:v>1.67</x:v>
+      </x:c>
+      <x:c r="X16" s="6">
+        <x:v>1635</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="s">
-        <x:v>103</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B17" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C17" s="2" t="s">
-        <x:v>104</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="D17" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E17" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F17" s="2" t="s">
-        <x:v>55</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G17" s="3">
         <x:v>1974</x:v>
@@ -1906,39 +2079,48 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R17" s="2" t="s">
-        <x:v>105</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="S17" s="2" t="s">
-        <x:v>106</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="T17" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U17" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="V17" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="W17" s="5">
+        <x:v>1.68</x:v>
+      </x:c>
+      <x:c r="X17" s="6">
+        <x:v>1342</x:v>
+      </x:c>
+      <x:c r="Y17" s="7">
+        <x:v>1.3158</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="s">
-        <x:v>107</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B18" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C18" s="2" t="s">
-        <x:v>108</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="D18" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E18" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F18" s="2" t="s">
-        <x:v>55</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G18" s="3">
         <x:v>1994</x:v>
@@ -1959,45 +2141,54 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R18" s="2" t="s">
-        <x:v>109</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="S18" s="2" t="s">
-        <x:v>110</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="T18" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U18" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="V18" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="W18" s="5">
+        <x:v>2.12</x:v>
+      </x:c>
+      <x:c r="X18" s="6">
+        <x:v>1567</x:v>
+      </x:c>
+      <x:c r="Y18" s="7">
+        <x:v>2.6667</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2" t="s">
-        <x:v>111</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B19" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C19" s="2" t="s">
-        <x:v>112</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="D19" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E19" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F19" s="2" t="s">
-        <x:v>113</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="G19" s="3">
         <x:v>2019</x:v>
       </x:c>
       <x:c r="H19" s="2" t="s">
-        <x:v>114</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="I19" s="4">
         <x:v>902</x:v>
@@ -2018,42 +2209,51 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="Q19" s="2" t="s">
-        <x:v>115</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="R19" s="2" t="s">
-        <x:v>116</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="S19" s="2" t="s">
-        <x:v>117</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="T19" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U19" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V19" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="W19" s="5">
+        <x:v>2.19</x:v>
+      </x:c>
+      <x:c r="X19" s="6">
+        <x:v>1977</x:v>
+      </x:c>
+      <x:c r="Y19" s="7">
+        <x:v>3.6458</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2" t="s">
-        <x:v>118</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B20" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C20" s="2" t="s">
-        <x:v>119</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="D20" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E20" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F20" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G20" s="3">
         <x:v>1971</x:v>
@@ -2074,39 +2274,45 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R20" s="2" t="s">
-        <x:v>120</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="S20" s="2" t="s">
-        <x:v>121</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="T20" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U20" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V20" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W20" s="5">
+        <x:v>1.71</x:v>
+      </x:c>
+      <x:c r="X20" s="6">
+        <x:v>1303</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="2" t="s">
-        <x:v>122</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B21" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C21" s="2" t="s">
-        <x:v>123</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="D21" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E21" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F21" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G21" s="3">
         <x:v>1999</x:v>
@@ -2130,39 +2336,48 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R21" s="2" t="s">
-        <x:v>124</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="S21" s="2" t="s">
-        <x:v>125</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="T21" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U21" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V21" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W21" s="5">
+        <x:v>2.27</x:v>
+      </x:c>
+      <x:c r="X21" s="6">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="Y21" s="7">
+        <x:v>1.9481</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="s">
-        <x:v>126</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B22" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C22" s="2" t="s">
-        <x:v>127</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D22" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E22" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F22" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G22" s="3">
         <x:v>1987</x:v>
@@ -2186,39 +2401,48 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R22" s="2" t="s">
-        <x:v>128</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="S22" s="2" t="s">
-        <x:v>129</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="T22" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U22" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V22" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W22" s="5">
+        <x:v>1.46</x:v>
+      </x:c>
+      <x:c r="X22" s="6">
+        <x:v>1389</x:v>
+      </x:c>
+      <x:c r="Y22" s="7">
+        <x:v>7.9365</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="2" t="s">
-        <x:v>130</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B23" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C23" s="2" t="s">
-        <x:v>131</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="D23" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E23" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F23" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G23" s="3">
         <x:v>1991</x:v>
@@ -2239,45 +2463,54 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R23" s="2" t="s">
-        <x:v>132</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="S23" s="2" t="s">
-        <x:v>133</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="T23" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U23" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V23" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W23" s="5">
+        <x:v>2.26</x:v>
+      </x:c>
+      <x:c r="X23" s="6">
+        <x:v>1790</x:v>
+      </x:c>
+      <x:c r="Y23" s="7">
+        <x:v>5.9524</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="2" t="s">
-        <x:v>134</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B24" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C24" s="2" t="s">
-        <x:v>135</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="D24" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E24" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F24" s="2" t="s">
-        <x:v>136</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="G24" s="3">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="H24" s="2" t="s">
-        <x:v>67</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I24" s="4">
         <x:v>896</x:v>
@@ -2301,45 +2534,54 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R24" s="2" t="s">
-        <x:v>137</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="S24" s="2" t="s">
-        <x:v>138</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="T24" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U24" s="2" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="V24" s="2" t="s">
-        <x:v>139</x:v>
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="W24" s="5">
+        <x:v>2.45</x:v>
+      </x:c>
+      <x:c r="X24" s="6">
+        <x:v>2196</x:v>
+      </x:c>
+      <x:c r="Y24" s="7">
+        <x:v>3.2847</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="2" t="s">
-        <x:v>140</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B25" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C25" s="2" t="s">
-        <x:v>141</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="D25" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E25" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F25" s="2" t="s">
-        <x:v>142</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="G25" s="3">
         <x:v>2018</x:v>
       </x:c>
       <x:c r="H25" s="2" t="s">
-        <x:v>143</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="I25" s="4">
         <x:v>942</x:v>
@@ -2357,48 +2599,57 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="Q25" s="2" t="s">
-        <x:v>144</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="R25" s="2" t="s">
-        <x:v>145</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="S25" s="2" t="s">
-        <x:v>146</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="T25" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U25" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V25" s="2" t="s">
-        <x:v>147</x:v>
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="W25" s="5">
+        <x:v>1.67</x:v>
+      </x:c>
+      <x:c r="X25" s="6">
+        <x:v>1572</x:v>
+      </x:c>
+      <x:c r="Y25" s="7">
+        <x:v>1.9231</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="2" t="s">
-        <x:v>148</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B26" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C26" s="2" t="s">
-        <x:v>149</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D26" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E26" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F26" s="2" t="s">
-        <x:v>150</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="G26" s="3">
         <x:v>2021</x:v>
       </x:c>
       <x:c r="H26" s="2" t="s">
-        <x:v>151</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="I26" s="4">
         <x:v>818</x:v>
@@ -2419,48 +2670,57 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q26" s="2" t="s">
-        <x:v>152</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="R26" s="2" t="s">
-        <x:v>153</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="S26" s="2" t="s">
-        <x:v>154</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="T26" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U26" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="V26" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="W26" s="5">
+        <x:v>2.47</x:v>
+      </x:c>
+      <x:c r="X26" s="6">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="Y26" s="7">
+        <x:v>6.3291</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="2" t="s">
-        <x:v>155</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B27" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C27" s="2" t="s">
-        <x:v>156</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="D27" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E27" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F27" s="2" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G27" s="3">
         <x:v>2016</x:v>
       </x:c>
       <x:c r="H27" s="2" t="s">
-        <x:v>157</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="I27" s="4">
         <x:v>874</x:v>
@@ -2478,48 +2738,57 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="Q27" s="2" t="s">
-        <x:v>158</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="R27" s="2" t="s">
-        <x:v>158</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="S27" s="2" t="s">
-        <x:v>159</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="T27" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U27" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V27" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W27" s="5">
+        <x:v>2.54</x:v>
+      </x:c>
+      <x:c r="X27" s="6">
+        <x:v>2219</x:v>
+      </x:c>
+      <x:c r="Y27" s="7">
+        <x:v>1.7422</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="2" t="s">
-        <x:v>160</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B28" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C28" s="2" t="s">
-        <x:v>161</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D28" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E28" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F28" s="2" t="s">
-        <x:v>76</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="G28" s="3">
         <x:v>2017</x:v>
       </x:c>
       <x:c r="H28" s="2" t="s">
-        <x:v>162</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="I28" s="4">
         <x:v>1012</x:v>
@@ -2540,42 +2809,51 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q28" s="2" t="s">
-        <x:v>163</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="R28" s="2" t="s">
-        <x:v>163</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="S28" s="2" t="s">
-        <x:v>164</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="T28" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U28" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="V28" s="2" t="s">
-        <x:v>165</x:v>
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="W28" s="5">
+        <x:v>2.25</x:v>
+      </x:c>
+      <x:c r="X28" s="6">
+        <x:v>2282</x:v>
+      </x:c>
+      <x:c r="Y28" s="7">
+        <x:v>2.4691</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="2" t="s">
-        <x:v>166</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B29" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C29" s="2" t="s">
-        <x:v>167</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="D29" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E29" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F29" s="2" t="s">
-        <x:v>168</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="G29" s="3">
         <x:v>1994</x:v>
@@ -2599,39 +2877,48 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R29" s="2" t="s">
-        <x:v>169</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="S29" s="2" t="s">
-        <x:v>170</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="T29" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U29" s="2" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="V29" s="2" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="W29" s="5">
+        <x:v>2.13</x:v>
+      </x:c>
+      <x:c r="X29" s="6">
+        <x:v>2075</x:v>
+      </x:c>
+      <x:c r="Y29" s="7">
+        <x:v>0.7874</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="2" t="s">
-        <x:v>171</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B30" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C30" s="2" t="s">
-        <x:v>172</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="D30" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E30" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F30" s="2" t="s">
-        <x:v>173</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="G30" s="3">
         <x:v>1985</x:v>
@@ -2652,39 +2939,48 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R30" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="S30" s="2" t="s">
-        <x:v>175</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="T30" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U30" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V30" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W30" s="5">
+        <x:v>2.58</x:v>
+      </x:c>
+      <x:c r="X30" s="6">
+        <x:v>2077</x:v>
+      </x:c>
+      <x:c r="Y30" s="7">
+        <x:v>3.1915</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="2" t="s">
-        <x:v>176</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B31" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C31" s="2" t="s">
-        <x:v>177</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="D31" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E31" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F31" s="2" t="s">
-        <x:v>35</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="G31" s="3">
         <x:v>1976</x:v>
@@ -2705,39 +3001,48 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R31" s="2" t="s">
-        <x:v>178</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="S31" s="2" t="s">
-        <x:v>179</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="T31" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U31" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V31" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="W31" s="5">
+        <x:v>1.94</x:v>
+      </x:c>
+      <x:c r="X31" s="6">
+        <x:v>1440</x:v>
+      </x:c>
+      <x:c r="Y31" s="7">
+        <x:v>1.7857</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="2" t="s">
-        <x:v>180</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B32" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C32" s="2" t="s">
-        <x:v>181</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="D32" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E32" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F32" s="2" t="s">
-        <x:v>182</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="G32" s="3">
         <x:v>1969</x:v>
@@ -2761,39 +3066,48 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="R32" s="2" t="s">
-        <x:v>183</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="S32" s="2" t="s">
-        <x:v>184</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="T32" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U32" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V32" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="W32" s="5">
+        <x:v>2.22</x:v>
+      </x:c>
+      <x:c r="X32" s="6">
+        <x:v>1598</x:v>
+      </x:c>
+      <x:c r="Y32" s="7">
+        <x:v>1.875</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="2" t="s">
-        <x:v>185</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="B33" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C33" s="2" t="s">
-        <x:v>186</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="D33" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E33" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F33" s="2" t="s">
-        <x:v>55</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G33" s="3">
         <x:v>1969</x:v>
@@ -2817,39 +3131,45 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R33" s="2" t="s">
-        <x:v>187</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="S33" s="2" t="s">
-        <x:v>188</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="T33" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U33" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="V33" s="2" t="s">
-        <x:v>59</x:v>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="W33" s="5">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="X33" s="6">
+        <x:v>1491</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="2" t="s">
-        <x:v>189</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="B34" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C34" s="2" t="s">
-        <x:v>190</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="D34" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E34" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F34" s="2" t="s">
-        <x:v>35</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="G34" s="3">
         <x:v>1975</x:v>
@@ -2861,16 +3181,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="R34" s="2" t="s">
-        <x:v>191</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="T34" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="U34" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="V34" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="Y34" s="7">
+        <x:v>2.5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3139,13 +3462,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6AEE8859-66E2-498A-9866-148E9EC65562}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA4396A4-7C9D-4AFC-8483-458FE13AB7DF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4070FF6C-F403-43F1-A0AF-EB1E20C43024}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEBA0F10-0669-4F9E-979A-D8053C847504}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2748C0FD-DFD3-4724-9984-3DC000A8D463}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35B6E744-BA04-4A32-AD66-4A3B89C90CD6}"/>
 </file>
</xml_diff>